<commit_message>
Add FY2021 NABIL data: 2,166 employees, 135 branches
Extracted from NABIL Annual Report 2020-21:
- Employees: 2,166 (as of mid-July 2021)
- Branches: 135
- CAR: 12.77%

NABIL now has complete employee/branch data for FY2020-2025.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/DATA/04_operating_metrics.xlsx
+++ b/DATA/04_operating_metrics.xlsx
@@ -2849,6 +2849,12 @@
       <c r="C57">
         <v>2021</v>
       </c>
+      <c r="D57">
+        <v>135</v>
+      </c>
+      <c r="E57">
+        <v>2166</v>
+      </c>
       <c r="F57">
         <v>148</v>
       </c>

</xml_diff>